<commit_message>
Adjusted from PR feedback
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/negative/01/data/new-rule-negative-1.xlsx
+++ b/rules/NEW-RULE/negative/01/data/new-rule-negative-1.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\NEW-RULE\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D6152E-3ADB-4A2D-AD48-A074454DF7DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26F556D-F99C-4A7B-8C5C-EC88C6CBEA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1755" yWindow="2460" windowWidth="26790" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" r:id="rId3"/>
-    <sheet name="ts.xpt" sheetId="4" r:id="rId4"/>
-    <sheet name="dm.xpt" sheetId="5" r:id="rId5"/>
+    <sheet name="Validation" sheetId="5" r:id="rId3"/>
+    <sheet name="ts.xpt" sheetId="3" r:id="rId4"/>
+    <sheet name="dm.xpt" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="151">
   <si>
     <t>Product</t>
   </si>
@@ -50,54 +50,27 @@
     <t>Trial Summary Parameters</t>
   </si>
   <si>
-    <t>Error group</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Error level</t>
-  </si>
-  <si>
-    <t>Row num</t>
-  </si>
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>Error value</t>
-  </si>
-  <si>
-    <t>Record</t>
+    <t>STUDYID</t>
+  </si>
+  <si>
+    <t>DOMAIN</t>
+  </si>
+  <si>
+    <t>TSSEQ</t>
+  </si>
+  <si>
+    <t>TSGRPID</t>
   </si>
   <si>
     <t>TSPARMCD</t>
   </si>
   <si>
-    <t>ADDL</t>
+    <t>TSPARM</t>
   </si>
   <si>
     <t>TSVAL</t>
   </si>
   <si>
-    <t>Val 2</t>
-  </si>
-  <si>
-    <t>STUDYID</t>
-  </si>
-  <si>
-    <t>DOMAIN</t>
-  </si>
-  <si>
-    <t>TSSEQ</t>
-  </si>
-  <si>
-    <t>TSGRPID</t>
-  </si>
-  <si>
-    <t>TSPARM</t>
-  </si>
-  <si>
     <t>TSVALNF</t>
   </si>
   <si>
@@ -179,31 +152,31 @@
     <t>TS</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Additional</t>
-  </si>
-  <si>
     <t>CDISC</t>
   </si>
   <si>
     <t>2018-12-21</t>
   </si>
   <si>
-    <t>CURTRT</t>
-  </si>
-  <si>
-    <t>Current Treatment</t>
-  </si>
-  <si>
-    <t>DRUG A1</t>
-  </si>
-  <si>
     <t>dm.xpt</t>
   </si>
   <si>
     <t>Demographics</t>
+  </si>
+  <si>
+    <t>SSDTC</t>
+  </si>
+  <si>
+    <t>2018-04-15</t>
+  </si>
+  <si>
+    <t>Study Start Date</t>
   </si>
   <si>
     <t>USUBJID</t>
@@ -484,10 +457,28 @@
     <t>GRC</t>
   </si>
   <si>
-    <t>SSDTC</t>
-  </si>
-  <si>
-    <t>Study Start Date</t>
+    <t>Error group</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Error level</t>
+  </si>
+  <si>
+    <t>Row num</t>
+  </si>
+  <si>
+    <t>Variable</t>
+  </si>
+  <si>
+    <t>Error value</t>
+  </si>
+  <si>
+    <t>Record</t>
+  </si>
+  <si>
+    <t>$dm_rficdtc</t>
   </si>
 </sst>
 </file>
@@ -605,7 +596,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -633,9 +624,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1025,10 +1017,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1040,7 +1032,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26947DD5-A09A-423F-BFD3-C313010AFFB4}">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1050,22 +1042,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>8</v>
+        <v>143</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>9</v>
+        <v>144</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>11</v>
+        <v>146</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>12</v>
+        <v>147</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>13</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1076,16 +1068,16 @@
         <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="D2" s="2">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>152</v>
+        <v>12</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1096,24 +1088,35 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="D3" s="2">
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>112</v>
+        <v>14</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>149</v>
+      </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -1125,509 +1128,444 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:F1 A2:D2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" customWidth="1"/>
-    <col min="12" max="12" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="5">
-        <v>1</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>112</v>
-      </c>
       <c r="H5" s="5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G6" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" t="s">
-        <v>53</v>
-      </c>
-      <c r="K6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="5">
-        <v>3</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K4 A6:K7 A5:D5 H5:K5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K4 A5:D5 H5:K5" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7523059F-2EFA-410B-BAD8-A9C741619A6A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10521100-C481-40B4-95F5-06F7F9F64B06}">
   <dimension ref="A1:Z8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="T1" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="U1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="W1" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="X1" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="R1" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="S1" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="T1" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="U1" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="V1" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="W1" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="X1" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="Z1" s="6" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="M2" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="P2" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="Q2" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="R2" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="T2" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="V2" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="W2" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="X2" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="Y2" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Z2" s="8" t="s">
         <v>98</v>
-      </c>
-      <c r="R2" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="S2" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="U2" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="W2" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="X2" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="Y2" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z2" s="8" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="U3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="V3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="W3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="Z3" s="8" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
@@ -1712,262 +1650,262 @@
     </row>
     <row r="5" spans="1:26" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="K5" s="11"/>
       <c r="L5" s="12" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="M5" s="11" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="R5" s="11" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="S5" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="T5" s="11"/>
       <c r="U5" s="11" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="11" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="Y5" s="11"/>
       <c r="Z5" s="11" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="K6" s="11"/>
       <c r="L6" s="12" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="O6" s="11" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="P6" s="11" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="Q6" s="11" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="S6" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="T6" s="11"/>
       <c r="U6" s="11"/>
       <c r="V6" s="11"/>
       <c r="W6" s="11" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="X6" s="11" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="Y6" s="11"/>
       <c r="Z6" s="11" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
       <c r="I7" s="11" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="L7" s="11"/>
       <c r="M7" s="11" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="O7" s="11"/>
       <c r="P7" s="11" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="Q7" s="11" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="R7" s="11" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="S7" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="T7" s="11"/>
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
       <c r="X7" s="11" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="Y7" s="11"/>
       <c r="Z7" s="11" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="B8" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="P8" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="Q8" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="R8" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="S8" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="T8" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="U8" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="V8" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="W8" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="X8" s="11" t="s">
         <v>141</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="L8" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="O8" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="P8" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q8" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="R8" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="S8" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="T8" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="U8" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="V8" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="W8" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="X8" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="Y8" s="12"/>
       <c r="Z8" s="12" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>